<commit_message>
Add instant and backend sorting for shareholder data viewer
</commit_message>
<xml_diff>
--- a/data/output/parsed/Tech Mahindra_2017-18.xlsx
+++ b/data/output/parsed/Tech Mahindra_2017-18.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2026-03-15T21:36:18Z</t>
+          <t>2026-03-18T23:44:14Z</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-03-15T21:36:18Z</t>
+          <t>2026-03-18T23:44:14Z</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2026-03-15T21:36:18Z</t>
+          <t>2026-03-18T23:44:14Z</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-03-15T21:36:18Z</t>
+          <t>2026-03-18T23:44:14Z</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2026-03-15T21:36:18Z</t>
+          <t>2026-03-18T23:44:14Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement background task queue, SSE, and normalized DB schema; fix dashboard polling and upload status
</commit_message>
<xml_diff>
--- a/data/output/parsed/Tech Mahindra_2017-18.xlsx
+++ b/data/output/parsed/Tech Mahindra_2017-18.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2026-03-18T23:44:14Z</t>
+          <t>2026-03-19T20:46:22Z</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-03-18T23:44:14Z</t>
+          <t>2026-03-19T20:46:22Z</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2026-03-18T23:44:14Z</t>
+          <t>2026-03-19T20:46:22Z</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-03-18T23:44:14Z</t>
+          <t>2026-03-19T20:46:22Z</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2026-03-18T23:44:14Z</t>
+          <t>2026-03-19T20:46:22Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: robust DB schema for shareholders, align columns, drop/recreate table, update insert logic
</commit_message>
<xml_diff>
--- a/data/output/parsed/Tech Mahindra_2017-18.xlsx
+++ b/data/output/parsed/Tech Mahindra_2017-18.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2026-03-19T20:46:22Z</t>
+          <t>2026-03-19T23:53:16Z</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-03-19T20:46:22Z</t>
+          <t>2026-03-19T23:53:16Z</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2026-03-19T20:46:22Z</t>
+          <t>2026-03-19T23:53:16Z</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-03-19T20:46:22Z</t>
+          <t>2026-03-19T23:53:16Z</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2026-03-19T20:46:22Z</t>
+          <t>2026-03-19T23:53:16Z</t>
         </is>
       </c>
     </row>

</xml_diff>